<commit_message>
Improve schedule report data quality
</commit_message>
<xml_diff>
--- a/reports/weekly_report.xlsx
+++ b/reports/weekly_report.xlsx
@@ -446,7 +446,7 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="38" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>每年春季至暑期关注学校通知</t>
+          <t>2026年9月10日</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026年</t>
+          <t>2026年9月10日</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
@@ -1921,12 +1921,12 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>通常每年4月至6月启动</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>通常每年4月至10月</t>
+          <t>2025-05-27</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2491,11 +2491,7 @@
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>2009-20</t>
-        </is>
-      </c>
+      <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr">
         <is>
           <t>https://www.tiaozhanbei.net/article/15838/</t>
@@ -2615,7 +2611,7 @@
       <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>2025.11.03</t>
+          <t>2025.11.15</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2676,7 +2672,11 @@
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>6月1日</t>
+        </is>
+      </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
           <t>https://www.tiaozhanbei.net/rules</t>
@@ -2825,7 +2825,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="38" customWidth="1" min="8" max="8"/>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>每年春季至暑期关注学校通知</t>
+          <t>2026年9月10日</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026年</t>
+          <t>2026年9月10日</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
@@ -5292,12 +5292,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>通常每年4月至6月启动</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>通常每年4月至10月</t>
+          <t>2025-05-27</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -6285,11 +6285,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>2009-20</t>
-        </is>
-      </c>
+      <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr"/>
@@ -6487,7 +6483,7 @@
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2025.11.03</t>
+          <t>2025.11.15</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
@@ -6587,7 +6583,11 @@
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>6月1日</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>

</xml_diff>